<commit_message>
feat(sharadar): add the Sharadar data provider
Reads stocks, funds, fundamentals, dividends and splits through Sharadar's query API in batches of 30 identifiers, with retries, rate limit waits and per-identifier skips. Passes on data as Sharadar publishes it: split adjusted dividends only, as-reported fundamentals from their whole history, the reporting currency of the filings.
</commit_message>
<xml_diff>
--- a/templates/data_curator/Config/data_curator_parameters.xlsx
+++ b/templates/data_curator/Config/data_curator_parameters.xlsx
@@ -1719,13 +1719,13 @@
   <phoneticPr fontId="16"/>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B4:B5" xr:uid="{2E694D9E-5091-4438-84ED-E24E52EF7C10}">
-      <formula1>"FinancialModelingPrep,LsegWorkspace,YahooFinance,None"</formula1>
+      <formula1>"FinancialModelingPrep,LsegWorkspace,Sharadar,YahooFinance,None"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{24DE7AE5-DCAA-4E1E-AB0A-0B7231D19E90}">
-      <formula1>"FinancialModelingPrep,LsegWorkspace,YahooFinance"</formula1>
+      <formula1>"FinancialModelingPrep,LsegWorkspace,Sharadar,YahooFinance"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3" xr:uid="{6764D2B7-BDEA-47DC-8E6C-55F0307CCA1A}">
-      <formula1>"FinancialModelingPrep,LsegWorkspace,None"</formula1>
+      <formula1>"FinancialModelingPrep,LsegWorkspace,Sharadar,None"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>